<commit_message>
added History function to view from perspective
</commit_message>
<xml_diff>
--- a/testing.xlsx
+++ b/testing.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://analog-my.sharepoint.com/personal/jake_ciolfi_analog_com/Documents/3. Resources/Coding Projects/RCO_Scramble/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="169" documentId="11_F25DC773A252ABDACC1048BDC11F63425BDE58E3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8AE80B0E-EAE7-4BB8-9A9D-FA04EE6F7B89}"/>
+  <xr:revisionPtr revIDLastSave="183" documentId="11_F25DC773A252ABDACC1048BDC11F63425BDE58E3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3A9CC9F-139D-44CA-9076-D145FE29585E}"/>
   <bookViews>
-    <workbookView xWindow="43470" yWindow="2295" windowWidth="20415" windowHeight="9720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -59,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="24">
   <si>
     <t>Round</t>
   </si>
@@ -1503,4 +1504,386 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66A23499-349C-402E-B733-0E4257D1D5B6}">
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" t="str" cm="1">
+        <f t="array" ref="H5:H12">_xlfn._xlws.FILTER(B:B, A:A=H3)</f>
+        <v>W1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" t="str">
+        <v>W2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" t="str">
+        <v>W4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" t="str">
+        <v>W5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" t="str">
+        <v>W1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" t="s">
+        <v>19</v>
+      </c>
+      <c r="H10" t="str">
+        <v>W2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" t="str">
+        <v>W4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" t="s">
+        <v>22</v>
+      </c>
+      <c r="H12" t="str">
+        <v>W5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" t="s">
+        <v>22</v>
+      </c>
+      <c r="H14">
+        <f>COUNTA(H5:H12)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" t="s">
+        <v>19</v>
+      </c>
+      <c r="H15">
+        <f>COUNTA(_xlfn.UNIQUE(H5:H12))</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" t="s">
+        <v>21</v>
+      </c>
+      <c r="D23" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>